<commit_message>
incluindo planilha das matrizes de confusao
</commit_message>
<xml_diff>
--- a/interpretacao/tabela_comparativa_algoritmos.xlsx
+++ b/interpretacao/tabela_comparativa_algoritmos.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Métricas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrizes de Confusão" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1753,4 +1754,1215 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Quantidade Atributos</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Coleção</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Algoritmo</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Verdadeiros Negativos (VN)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Falsos Positivos (FP)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Falsos Negativos (FN)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Verdadeiros Positivos (VP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>treino_e_teste_1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Decision Tree</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>735</v>
+      </c>
+      <c r="E2" t="n">
+        <v>277</v>
+      </c>
+      <c r="F2" t="n">
+        <v>419</v>
+      </c>
+      <c r="G2" t="n">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>treino_e_teste_1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Naive Bayes</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>444</v>
+      </c>
+      <c r="E3" t="n">
+        <v>568</v>
+      </c>
+      <c r="F3" t="n">
+        <v>233</v>
+      </c>
+      <c r="G3" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>treino_e_teste_1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>705</v>
+      </c>
+      <c r="E4" t="n">
+        <v>307</v>
+      </c>
+      <c r="F4" t="n">
+        <v>394</v>
+      </c>
+      <c r="G4" t="n">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>treino_e_teste_1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>672</v>
+      </c>
+      <c r="E5" t="n">
+        <v>340</v>
+      </c>
+      <c r="F5" t="n">
+        <v>357</v>
+      </c>
+      <c r="G5" t="n">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>treino_e_teste_2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Decision Tree</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>718</v>
+      </c>
+      <c r="E6" t="n">
+        <v>294</v>
+      </c>
+      <c r="F6" t="n">
+        <v>424</v>
+      </c>
+      <c r="G6" t="n">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>treino_e_teste_2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Naive Bayes</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>419</v>
+      </c>
+      <c r="E7" t="n">
+        <v>593</v>
+      </c>
+      <c r="F7" t="n">
+        <v>189</v>
+      </c>
+      <c r="G7" t="n">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>treino_e_teste_2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>683</v>
+      </c>
+      <c r="E8" t="n">
+        <v>329</v>
+      </c>
+      <c r="F8" t="n">
+        <v>405</v>
+      </c>
+      <c r="G8" t="n">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>treino_e_teste_2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>722</v>
+      </c>
+      <c r="E9" t="n">
+        <v>290</v>
+      </c>
+      <c r="F9" t="n">
+        <v>408</v>
+      </c>
+      <c r="G9" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>treino_e_teste_3</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Decision Tree</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>657</v>
+      </c>
+      <c r="E10" t="n">
+        <v>355</v>
+      </c>
+      <c r="F10" t="n">
+        <v>413</v>
+      </c>
+      <c r="G10" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>treino_e_teste_3</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Naive Bayes</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>549</v>
+      </c>
+      <c r="E11" t="n">
+        <v>463</v>
+      </c>
+      <c r="F11" t="n">
+        <v>261</v>
+      </c>
+      <c r="G11" t="n">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>treino_e_teste_3</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>680</v>
+      </c>
+      <c r="E12" t="n">
+        <v>332</v>
+      </c>
+      <c r="F12" t="n">
+        <v>399</v>
+      </c>
+      <c r="G12" t="n">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>treino_e_teste_3</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>683</v>
+      </c>
+      <c r="E13" t="n">
+        <v>329</v>
+      </c>
+      <c r="F13" t="n">
+        <v>383</v>
+      </c>
+      <c r="G13" t="n">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>treino_e_teste_4</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Decision Tree</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>715</v>
+      </c>
+      <c r="E14" t="n">
+        <v>297</v>
+      </c>
+      <c r="F14" t="n">
+        <v>460</v>
+      </c>
+      <c r="G14" t="n">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>treino_e_teste_4</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Naive Bayes</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>669</v>
+      </c>
+      <c r="E15" t="n">
+        <v>343</v>
+      </c>
+      <c r="F15" t="n">
+        <v>372</v>
+      </c>
+      <c r="G15" t="n">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>treino_e_teste_4</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>693</v>
+      </c>
+      <c r="E16" t="n">
+        <v>319</v>
+      </c>
+      <c r="F16" t="n">
+        <v>441</v>
+      </c>
+      <c r="G16" t="n">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>treino_e_teste_4</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>725</v>
+      </c>
+      <c r="E17" t="n">
+        <v>287</v>
+      </c>
+      <c r="F17" t="n">
+        <v>425</v>
+      </c>
+      <c r="G17" t="n">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>treino_e_teste_5</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Decision Tree</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>668</v>
+      </c>
+      <c r="E18" t="n">
+        <v>344</v>
+      </c>
+      <c r="F18" t="n">
+        <v>412</v>
+      </c>
+      <c r="G18" t="n">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>treino_e_teste_5</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Naive Bayes</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>622</v>
+      </c>
+      <c r="E19" t="n">
+        <v>390</v>
+      </c>
+      <c r="F19" t="n">
+        <v>326</v>
+      </c>
+      <c r="G19" t="n">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>treino_e_teste_5</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>662</v>
+      </c>
+      <c r="E20" t="n">
+        <v>350</v>
+      </c>
+      <c r="F20" t="n">
+        <v>388</v>
+      </c>
+      <c r="G20" t="n">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>treino_e_teste_5</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>695</v>
+      </c>
+      <c r="E21" t="n">
+        <v>317</v>
+      </c>
+      <c r="F21" t="n">
+        <v>397</v>
+      </c>
+      <c r="G21" t="n">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>treino_e_teste_1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Decision Tree</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>608</v>
+      </c>
+      <c r="E22" t="n">
+        <v>404</v>
+      </c>
+      <c r="F22" t="n">
+        <v>413</v>
+      </c>
+      <c r="G22" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>treino_e_teste_1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Naive Bayes</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>493</v>
+      </c>
+      <c r="E23" t="n">
+        <v>519</v>
+      </c>
+      <c r="F23" t="n">
+        <v>246</v>
+      </c>
+      <c r="G23" t="n">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>treino_e_teste_1</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>686</v>
+      </c>
+      <c r="E24" t="n">
+        <v>326</v>
+      </c>
+      <c r="F24" t="n">
+        <v>399</v>
+      </c>
+      <c r="G24" t="n">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>treino_e_teste_1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>691</v>
+      </c>
+      <c r="E25" t="n">
+        <v>321</v>
+      </c>
+      <c r="F25" t="n">
+        <v>387</v>
+      </c>
+      <c r="G25" t="n">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>treino_e_teste_2</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Decision Tree</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>655</v>
+      </c>
+      <c r="E26" t="n">
+        <v>357</v>
+      </c>
+      <c r="F26" t="n">
+        <v>388</v>
+      </c>
+      <c r="G26" t="n">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>treino_e_teste_2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Naive Bayes</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>434</v>
+      </c>
+      <c r="E27" t="n">
+        <v>578</v>
+      </c>
+      <c r="F27" t="n">
+        <v>212</v>
+      </c>
+      <c r="G27" t="n">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>treino_e_teste_2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>689</v>
+      </c>
+      <c r="E28" t="n">
+        <v>323</v>
+      </c>
+      <c r="F28" t="n">
+        <v>378</v>
+      </c>
+      <c r="G28" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>treino_e_teste_2</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>688</v>
+      </c>
+      <c r="E29" t="n">
+        <v>324</v>
+      </c>
+      <c r="F29" t="n">
+        <v>389</v>
+      </c>
+      <c r="G29" t="n">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>treino_e_teste_3</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Decision Tree</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>626</v>
+      </c>
+      <c r="E30" t="n">
+        <v>386</v>
+      </c>
+      <c r="F30" t="n">
+        <v>389</v>
+      </c>
+      <c r="G30" t="n">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>treino_e_teste_3</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Naive Bayes</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>545</v>
+      </c>
+      <c r="E31" t="n">
+        <v>467</v>
+      </c>
+      <c r="F31" t="n">
+        <v>255</v>
+      </c>
+      <c r="G31" t="n">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>treino_e_teste_3</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>724</v>
+      </c>
+      <c r="E32" t="n">
+        <v>288</v>
+      </c>
+      <c r="F32" t="n">
+        <v>398</v>
+      </c>
+      <c r="G32" t="n">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>treino_e_teste_3</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>689</v>
+      </c>
+      <c r="E33" t="n">
+        <v>323</v>
+      </c>
+      <c r="F33" t="n">
+        <v>391</v>
+      </c>
+      <c r="G33" t="n">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>treino_e_teste_4</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Decision Tree</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>675</v>
+      </c>
+      <c r="E34" t="n">
+        <v>337</v>
+      </c>
+      <c r="F34" t="n">
+        <v>424</v>
+      </c>
+      <c r="G34" t="n">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>treino_e_teste_4</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Naive Bayes</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>552</v>
+      </c>
+      <c r="E35" t="n">
+        <v>460</v>
+      </c>
+      <c r="F35" t="n">
+        <v>270</v>
+      </c>
+      <c r="G35" t="n">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>treino_e_teste_4</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>687</v>
+      </c>
+      <c r="E36" t="n">
+        <v>325</v>
+      </c>
+      <c r="F36" t="n">
+        <v>407</v>
+      </c>
+      <c r="G36" t="n">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>treino_e_teste_4</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>699</v>
+      </c>
+      <c r="E37" t="n">
+        <v>313</v>
+      </c>
+      <c r="F37" t="n">
+        <v>420</v>
+      </c>
+      <c r="G37" t="n">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>treino_e_teste_5</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Decision Tree</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>628</v>
+      </c>
+      <c r="E38" t="n">
+        <v>384</v>
+      </c>
+      <c r="F38" t="n">
+        <v>417</v>
+      </c>
+      <c r="G38" t="n">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>treino_e_teste_5</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Naive Bayes</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>562</v>
+      </c>
+      <c r="E39" t="n">
+        <v>450</v>
+      </c>
+      <c r="F39" t="n">
+        <v>277</v>
+      </c>
+      <c r="G39" t="n">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>treino_e_teste_5</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>705</v>
+      </c>
+      <c r="E40" t="n">
+        <v>307</v>
+      </c>
+      <c r="F40" t="n">
+        <v>421</v>
+      </c>
+      <c r="G40" t="n">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>treino_e_teste_5</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>702</v>
+      </c>
+      <c r="E41" t="n">
+        <v>310</v>
+      </c>
+      <c r="F41" t="n">
+        <v>389</v>
+      </c>
+      <c r="G41" t="n">
+        <v>339</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
ajustes na planilha comparativa matriz de confusao
</commit_message>
<xml_diff>
--- a/interpretacao/tabela_comparativa_algoritmos.xlsx
+++ b/interpretacao/tabela_comparativa_algoritmos.xlsx
@@ -1783,22 +1783,22 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Verdadeiros Negativos (VN)</t>
+          <t>Verdadeiros Negativos (VN) [Real: Desmame, Previsto: Desmame]</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Falsos Positivos (FP)</t>
+          <t>Falsos Positivos (FP) [Real: Desmame, Previsto: Sucesso]</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Falsos Negativos (FN)</t>
+          <t>Falsos Negativos (FN) [Real: Sucesso, Previsto: Desmame]</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Verdadeiros Positivos (VP)</t>
+          <t>Verdadeiros Positivos (VP) [Real: Sucesso, Previsto: Sucesso]</t>
         </is>
       </c>
     </row>

</xml_diff>